<commit_message>
fix: paper fonte unica (gerador, 8 metodos, todos os dias) — captura os dias que faltavam (0x2 etc.)
</commit_message>
<xml_diff>
--- a/placares_manuais.xlsx
+++ b/placares_manuais.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:H216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4541,31 +4541,31 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Ind Medellin</t>
+          <t>Wuxi Wugou</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Ningbo Professional</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>12</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
@@ -4573,31 +4573,31 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Colon</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>12.5</v>
+        <v>6.2</v>
       </c>
       <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr"/>
@@ -4605,31 +4605,31 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Mansfield</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Sheff Utd</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
@@ -4637,31 +4637,31 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Bodrum Belediyesi Bodrumspor</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Novorizontino</t>
+          <t>Bursaspor</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G118" t="inlineStr"/>
       <c r="H118" t="inlineStr"/>
@@ -4669,31 +4669,31 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>JAPAN 1</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Botev Vratsa</t>
+          <t>Tokyo-V</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Botev Plovdiv</t>
+          <t>Kawasaki</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>9.199999999999999</v>
+        <v>19</v>
       </c>
       <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr"/>
@@ -4701,31 +4701,31 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ENGLAND 1</t>
+          <t>JAPAN 2</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Yamagata</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Tochigi Uva FC</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr"/>
@@ -4733,31 +4733,31 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Crotone</t>
+          <t>Wuxi Wugou</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Foggia</t>
+          <t>Ningbo Professional</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>15.5</v>
+        <v>19</v>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr"/>
@@ -4765,31 +4765,31 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>CZECH 1</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Banik Ostrava B</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Novorizontino</t>
+          <t>MAS Taborsko</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>9</v>
+        <v>18.5</v>
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr"/>
@@ -4797,31 +4797,31 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>FINLAND 1</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>FC Inter</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Macara</t>
+          <t>Lahti</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>10.5</v>
+        <v>19</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr"/>
@@ -4829,31 +4829,31 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>AUSTRIA 1</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>SV Ried</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Rapid Vienna</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>8.199999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr"/>
@@ -4861,31 +4861,31 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ROMANIA 1</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>ACS Petrolul 52</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
@@ -4893,31 +4893,31 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>FRANCE 2</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Reims</t>
+          <t>76 Igdir Belediyespor</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Annecy</t>
+          <t>Fatih Karagumruk Istanbul</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>9.199999999999999</v>
+        <v>18.5</v>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr"/>
@@ -4925,31 +4925,31 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>CHILE 2</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Crotone</t>
+          <t>Deportes Copiapo</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Foggia</t>
+          <t>San Luis</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>8.800000000000001</v>
+        <v>17.5</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="inlineStr"/>
@@ -4957,31 +4957,31 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>BELGIUM 1</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Antwerp</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Waasland-Beveren</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>6.6</v>
+        <v>18.5</v>
       </c>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr"/>
@@ -4989,31 +4989,31 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>CHILE 2</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>CSD Rangers</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>America MG</t>
+          <t>Curico Unido</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>7.6</v>
+        <v>20</v>
       </c>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr"/>
@@ -5021,31 +5021,31 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Brondby</t>
+          <t>America de Cali S.A</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Silkeborg</t>
+          <t>Atletico Nacional Medellin</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>13.5</v>
+        <v>18</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -5053,31 +5053,31 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Gimnasia Jujuy</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Tristan Suarez</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>10.5</v>
+        <v>6</v>
       </c>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
@@ -5085,31 +5085,31 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>POLAND 2</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Unia Skierniewice</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="F132" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
@@ -5117,31 +5117,31 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ROMANIA 1</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>ACS Sepsi OSK</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>America MG</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
@@ -5149,31 +5149,31 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>PORTUGAL 2</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Botev Vratsa</t>
+          <t>Lusitania Futebol Clube</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Botev Plovdiv</t>
+          <t>Porto B</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr"/>
@@ -5181,31 +5181,31 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>ROMANIA 1</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Celta Vigo B</t>
+          <t>ACS Sepsi OSK</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>FCSB</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>34</v>
+        <v>19.5</v>
       </c>
       <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr"/>
@@ -5213,31 +5213,31 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>VENEZUELA 1</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Lokomotiv Plovdiv</t>
+          <t>Rayo Zuliano</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Arda</t>
+          <t>Estudiantes de Merida</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G136" t="inlineStr"/>
       <c r="H136" t="inlineStr"/>
@@ -5245,31 +5245,31 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Leones FC</t>
+          <t>Ind Medellin</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Real Cartagena</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>34</v>
+        <v>10.5</v>
       </c>
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
@@ -5277,31 +5277,31 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>SWEDEN 2</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Boca Juniors de Cali</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Union Magdalena</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>16.5</v>
+        <v>32</v>
       </c>
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr"/>
@@ -5309,7 +5309,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5319,21 +5319,21 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Real Santander</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Amed Sportif Faaliyetler</t>
+          <t>Barranquilla</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>19.5</v>
+        <v>20</v>
       </c>
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
@@ -5341,7 +5341,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5351,21 +5351,21 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Botafogo FR</t>
+          <t>Ind Medellin</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Athletico-PR</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
@@ -5373,34 +5373,2434 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>CHILE 2</t>
+          <t>PARAGUAY CUP</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>San Luis</t>
+          <t>Sportivo Iteno</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Santiago Wanderers</t>
+          <t>Guarani (Par)</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>18.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>COPA SUDAMERICANA</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>ARGENTINA CUP</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Atl Tucuman</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>CA Independiente</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>27</v>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>COPA SUDAMERICANA</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Cienciano</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Botafogo FR</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>19</v>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>JAPAN 1</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Tokyo-V</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Kashiwa</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>25</v>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CHINA 1</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Qingdao Youth Island</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Chongqing Tonglianglong</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>SAUDI ARABIA 1</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>NEOM Sports Club</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Al-Feiha</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>20</v>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ROMANIA 1</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Arges Pitesti</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Farul Constanta</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>FRANCE 2</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Dijon</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Pau</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>PARAGUAY 1</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Deportivo Recoleta</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Club 2 de Mayo de Pedro Juan</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Quilmes</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>JAPAN 1</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Urawa</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Hiroshima</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>25</v>
+      </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>JAPAN 2</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>FC Imabari</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Omiya</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>34</v>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>JAPAN 1</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Fukuoka</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Cerezo Osaka</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>18</v>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>JAPAN 1</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Kobe</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>FC Tokyo</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>19</v>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>JAPAN 2</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Sapporo</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>19</v>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>JAPAN 2</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Shonan</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Yamagata</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>20</v>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>SOUTH KOREA 1</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>FC Seoul</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Daejeon Citizen</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>17</v>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>ENGLAND 3</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Leyton Orient</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Sheff Wed</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>17</v>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Alverca</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Club Football Estrela</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>18</v>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PORTUGAL 2</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Sporting Lisbon B</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Chaves</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>18</v>
+      </c>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>CZECH 1</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>MAS Taborsko</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>SFC Opava</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>19</v>
+      </c>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>ENGLAND 2</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Sheff Utd</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Birmingham</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>ROMANIA 1</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Rapid Bucharest</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Dinamo Bucharest</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>18</v>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>VENEZUELA 1</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Estudiantes de Merida</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Academia Anzoategui FC</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>20</v>
+      </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>CHILE 1</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Everton De Vina</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Audax Italiano</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Tristan Suarez</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>ARGENTINA 2</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Gimnasia Jujuy</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Chaco For Ever</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>ROMANIA 1</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>22</v>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>PARAGUAY 1</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Sportivo Luqueno</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>24</v>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>SOUTH KOREA 1</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Ulsan Hyundai Horang-i</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Gangwon</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>17</v>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>CHINA 1</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Nanjing City</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Jiangxi Dingnan United</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>19</v>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>DENMARK 1</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>AC Horsens</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>20</v>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>PORTUGAL 2</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Amarante</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Lusitania Futebol Clube</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>20</v>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>CD Nacional Funchal</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Estoril Praia</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>16</v>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>ROMANIA 1</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Universitatea Craiova</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>BELGIUM 1</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Yellow-Red Mechelen</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>ROMANIA 1</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>FC Hunedoara</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>CFR Cluj</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>18</v>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>PARAGUAY 1</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Sportivo Luqueno</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>19</v>
+      </c>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>BRAZIL 1</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>EC Vitoria Salvador</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Botafogo FR</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>MEXICO 1</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Necaxa</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Leon</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>MEXICO 1</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Necaxa</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Leon</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>17</v>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>MEXICO 1</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Leon</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ECUADOR 1</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Deportivo Cuenca</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>20</v>
+      </c>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>CHILE 1</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Audax Italiano</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Union La Calera</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>18</v>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>USA 1</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>FC Dallas</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>USA 1</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Los Angeles FC</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Portland Timbers</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>13</v>
+      </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Lay Draw</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>MEXICO 1</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Puebla</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Santos Laguna</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>SOUTH KOREA 1</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>FC Anyang</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>FC Seoul</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>22</v>
+      </c>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Lay 0x0</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>SPAIN 1</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Lay 0x0</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>12</v>
+      </c>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Lay 0x0</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>America MG</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>BULGARIA 1</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Botev Vratsa</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Botev Plovdiv</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>ENGLAND 1</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>12</v>
+      </c>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>ITALY 3</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Crotone</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Foggia</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>9</v>
+      </c>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Lay 0x1</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>ECUADOR 1</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Libertad FC</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Macara</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>ITALY 1</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Lazio</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>FRANCE 2</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Reims</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Annecy</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>ITALY 3</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Crotone</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Foggia</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Lay 1x0</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>America MG</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>DENMARK 1</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Brondby</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Silkeborg</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>SPAIN 1</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>PORTUGAL 1</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Casa Pia</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>11</v>
+      </c>
+      <c r="G207" t="inlineStr"/>
+      <c r="H207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Lay 2x0</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Sport Recife</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>America MG</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>10</v>
+      </c>
+      <c r="G208" t="inlineStr"/>
+      <c r="H208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>BULGARIA 1</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Botev Vratsa</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Botev Plovdiv</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>29</v>
+      </c>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>SPAIN 2</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Celta Vigo B</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>FC Andorra</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>34</v>
+      </c>
+      <c r="G210" t="inlineStr"/>
+      <c r="H210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>BULGARIA 1</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Lokomotiv Plovdiv</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Arda</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>28</v>
+      </c>
+      <c r="G211" t="inlineStr"/>
+      <c r="H211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Lay 0x3</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>COLOMBIA 2</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Leones FC</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Real Cartagena</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>34</v>
+      </c>
+      <c r="G212" t="inlineStr"/>
+      <c r="H212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>SWEDEN 2</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Ostersunds FK</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Ljungskile</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>TURKEY 1</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Kocaelispor</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Amed Sportif Faaliyetler</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>BRAZIL 1</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Botafogo FR</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Athletico-PR</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>18</v>
+      </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>CHILE 2</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>San Luis</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Santiago Wanderers</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: placar Kalamata 2-3 Aris (coletor perdeu gol no acrescimo); manual agora tem prioridade sobre coletor/base
</commit_message>
<xml_diff>
--- a/placares_manuais.xlsx
+++ b/placares_manuais.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H216"/>
+  <dimension ref="A1:H218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6989,63 +6989,61 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Lay 1x0</t>
-        </is>
-      </c>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr"/>
       <c r="C183" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>GREECE 1</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Wuxi Wugou</t>
+          <t>Kalamata</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Ningbo Professional</t>
-        </is>
-      </c>
-      <c r="F183" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="n">
+        <v>2</v>
+      </c>
+      <c r="H183" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Wuxi Wugou</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Ningbo Professional</t>
+          <t>Macara</t>
         </is>
       </c>
       <c r="F184" t="n">
-        <v>19</v>
+        <v>10.5</v>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr"/>
@@ -7053,31 +7051,31 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Ind Medellin</t>
+          <t>Leones FC</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Real Cartagena</t>
         </is>
       </c>
       <c r="F185" t="n">
-        <v>10.5</v>
+        <v>34</v>
       </c>
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr"/>
@@ -7085,31 +7083,31 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x0</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Boca Juniors de Cali</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Union Magdalena</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F186" t="n">
-        <v>32</v>
+        <v>12.5</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
@@ -7117,31 +7115,31 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x0</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Real Santander</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Barranquilla</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="F187" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
@@ -7149,31 +7147,31 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Ind Medellin</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Millonarios</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="F188" t="n">
-        <v>19.5</v>
+        <v>11</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr"/>
@@ -7181,7 +7179,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -7191,21 +7189,21 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>COPA SUDAMERICANA</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>River Plate</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F189" t="n">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
@@ -7213,31 +7211,31 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F190" t="n">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
@@ -7245,31 +7243,31 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F191" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
@@ -7277,31 +7275,31 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="F192" t="n">
-        <v>12.5</v>
+        <v>11</v>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr"/>
@@ -7309,31 +7307,31 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="F193" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr"/>
@@ -7341,31 +7339,31 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>PARAGUAY CUP</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Sol de America</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>America MG</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F194" t="n">
-        <v>15.5</v>
+        <v>7.8</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr"/>
@@ -7373,7 +7371,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -7383,21 +7381,21 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Botev Vratsa</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Botev Plovdiv</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="F195" t="n">
-        <v>9.199999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
@@ -7405,7 +7403,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -7415,21 +7413,21 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ENGLAND 1</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="F196" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr"/>
@@ -7437,31 +7435,31 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Crotone</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Foggia</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F197" t="n">
-        <v>15.5</v>
+        <v>9.4</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
@@ -7469,31 +7467,31 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Novorizontino</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="F198" t="n">
-        <v>9</v>
+        <v>6.8</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr"/>
@@ -7501,31 +7499,31 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Atletico GO</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Macara</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="F199" t="n">
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr"/>
@@ -7533,7 +7531,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -7543,21 +7541,21 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>ITALY 1</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="F200" t="n">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
@@ -7565,31 +7563,31 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>FRANCE 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Reims</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Annecy</t>
+          <t>Leicester</t>
         </is>
       </c>
       <c r="F201" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
@@ -7597,31 +7595,31 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>ITALY 3</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Crotone</t>
+          <t>Al-Ettifaq</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Foggia</t>
+          <t>Al Nassr</t>
         </is>
       </c>
       <c r="F202" t="n">
-        <v>8.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
@@ -7629,31 +7627,31 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Blackpool</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Lincoln</t>
         </is>
       </c>
       <c r="F203" t="n">
-        <v>6.6</v>
+        <v>15.5</v>
       </c>
       <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr"/>
@@ -7661,31 +7659,31 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>America MG</t>
+          <t>Coventry</t>
         </is>
       </c>
       <c r="F204" t="n">
-        <v>7.6</v>
+        <v>11.5</v>
       </c>
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr"/>
@@ -7693,31 +7691,31 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Brondby</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Silkeborg</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="F205" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr"/>
@@ -7725,31 +7723,31 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F206" t="n">
-        <v>10.5</v>
+        <v>29</v>
       </c>
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr"/>
@@ -7757,31 +7755,31 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>PORTUGAL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Gil Vicente</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="F207" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr"/>
@@ -7789,31 +7787,31 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>PARAGUAY CUP</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Sol de America</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>America MG</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F208" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr"/>
@@ -7821,31 +7819,31 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>ROMANIA 2</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Botev Vratsa</t>
+          <t>Unirea Slobozia</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Botev Plovdiv</t>
+          <t>FC Metaloglobus Bucuresti</t>
         </is>
       </c>
       <c r="F209" t="n">
-        <v>29</v>
+        <v>18.5</v>
       </c>
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr"/>
@@ -7853,31 +7851,31 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>SPAIN 2</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Celta Vigo B</t>
+          <t>Al-Taawoun Buraidah</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Al-Feiha</t>
         </is>
       </c>
       <c r="F210" t="n">
-        <v>34</v>
+        <v>18.5</v>
       </c>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
@@ -7885,31 +7883,31 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Lokomotiv Plovdiv</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Arda</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F211" t="n">
-        <v>28</v>
+        <v>17.5</v>
       </c>
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr"/>
@@ -7917,31 +7915,31 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 2x2</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Leones FC</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Real Cartagena</t>
+          <t>Shrewsbury</t>
         </is>
       </c>
       <c r="F212" t="n">
-        <v>34</v>
+        <v>19.5</v>
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
@@ -7949,7 +7947,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -7959,21 +7957,21 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>SWEDEN 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F213" t="n">
-        <v>16.5</v>
+        <v>19.5</v>
       </c>
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
@@ -7981,7 +7979,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -7991,21 +7989,21 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>TURKEY 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Kocaelispor</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Amed Sportif Faaliyetler</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F214" t="n">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr"/>
@@ -8013,7 +8011,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -8023,21 +8021,21 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>BRAZIL 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Botafogo FR</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Athletico-PR</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="F215" t="n">
-        <v>18</v>
+        <v>17.5</v>
       </c>
       <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr"/>
@@ -8045,7 +8043,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -8055,24 +8053,88 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>CHILE 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>San Luis</t>
+          <t>Nottm Forest</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Santiago Wanderers</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="F216" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>PARAGUAY CUP</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>General Caballero</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Rubio Nu</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>18</v>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>SPAIN 1</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Betis</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>18</v>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: placares Sudtirol 1-0 (Lay 1x0 RED) e Queens Park 0-2 (Lay 0x1 GREEN) - coletor perdeu gol tardio; varredura de discordancias
</commit_message>
<xml_diff>
--- a/placares_manuais.xlsx
+++ b/placares_manuais.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H218"/>
+  <dimension ref="A1:H222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7019,95 +7019,91 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Lay 0x1</t>
-        </is>
-      </c>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr"/>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>ITALY 2</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Libertad FC</t>
+          <t>Sudtirol</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Macara</t>
-        </is>
-      </c>
-      <c r="F184" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
+          <t>Entella</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="n">
+        <v>1</v>
+      </c>
+      <c r="H184" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Lay 0x3</t>
-        </is>
-      </c>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr"/>
       <c r="C185" t="inlineStr">
         <is>
-          <t>COLOMBIA 2</t>
+          <t>SCOTLAND 2</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Leones FC</t>
+          <t>Queens Park</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Real Cartagena</t>
-        </is>
-      </c>
-      <c r="F185" t="n">
-        <v>34</v>
-      </c>
-      <c r="G185" t="inlineStr"/>
-      <c r="H185" t="inlineStr"/>
+          <t>Stenhousemuir</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>PORTUGAL 1</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Gil Vicente</t>
         </is>
       </c>
       <c r="F186" t="n">
-        <v>12.5</v>
+        <v>7.6</v>
       </c>
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr"/>
@@ -7115,31 +7111,31 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Lay 0x0</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>PORTUGAL 1</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Gil Vicente</t>
         </is>
       </c>
       <c r="F187" t="n">
-        <v>12</v>
+        <v>9.6</v>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr"/>
@@ -7147,7 +7143,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -7157,21 +7153,21 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Libertad FC</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Macara</t>
         </is>
       </c>
       <c r="F188" t="n">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr"/>
@@ -7179,31 +7175,31 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>COLOMBIA 2</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Cambridge Utd</t>
+          <t>Leones FC</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Real Cartagena</t>
         </is>
       </c>
       <c r="F189" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr"/>
@@ -7216,7 +7212,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 0x0</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -7226,16 +7222,16 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F190" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr"/>
@@ -7248,26 +7244,26 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 0x0</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="F191" t="n">
-        <v>9.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
@@ -7290,12 +7286,12 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Birmingham</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -7317,17 +7313,17 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -7349,21 +7345,21 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>PARAGUAY CUP</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Sol de America</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Sportivo Trinidense</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F194" t="n">
-        <v>7.8</v>
+        <v>10</v>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr"/>
@@ -7381,21 +7377,21 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ARGENTINA 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F195" t="n">
-        <v>11.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr"/>
@@ -7413,17 +7409,17 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Birmingham</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -7440,26 +7436,26 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>SPAIN 1</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="F197" t="n">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr"/>
@@ -7472,26 +7468,26 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>ARGENTINA 2</t>
+          <t>PARAGUAY CUP</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Deportivo Madryn</t>
+          <t>Sol de America</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Godoy Cruz</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F198" t="n">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr"/>
@@ -7504,26 +7500,26 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Atletico GO</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="F199" t="n">
-        <v>8</v>
+        <v>11.5</v>
       </c>
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr"/>
@@ -7536,7 +7532,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x1</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -7555,7 +7551,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>8.6</v>
+        <v>11</v>
       </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr"/>
@@ -7568,7 +7564,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Lay 2x0</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -7578,16 +7574,16 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Leicester</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F201" t="n">
-        <v>10.5</v>
+        <v>9.4</v>
       </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr"/>
@@ -7600,26 +7596,26 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>ARGENTINA 2</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Al-Ettifaq</t>
+          <t>Deportivo Madryn</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Al Nassr</t>
+          <t>Godoy Cruz</t>
         </is>
       </c>
       <c r="F202" t="n">
-        <v>12.5</v>
+        <v>6.8</v>
       </c>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
@@ -7632,26 +7628,26 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Blackpool</t>
+          <t>Atletico GO</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Lincoln</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="F203" t="n">
-        <v>15.5</v>
+        <v>8</v>
       </c>
       <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr"/>
@@ -7664,26 +7660,26 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>BRAZIL 2</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Coventry</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="F204" t="n">
-        <v>11.5</v>
+        <v>8.6</v>
       </c>
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr"/>
@@ -7696,7 +7692,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Lay 0x2</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -7706,16 +7702,16 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Leyton Orient</t>
+          <t>Leicester</t>
         </is>
       </c>
       <c r="F205" t="n">
-        <v>15</v>
+        <v>10.5</v>
       </c>
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr"/>
@@ -7728,26 +7724,26 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Cambridge Utd</t>
+          <t>Al-Ettifaq</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Al Nassr</t>
         </is>
       </c>
       <c r="F206" t="n">
-        <v>29</v>
+        <v>12.5</v>
       </c>
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr"/>
@@ -7760,7 +7756,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -7770,16 +7766,16 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Blackpool</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Leyton Orient</t>
+          <t>Lincoln</t>
         </is>
       </c>
       <c r="F207" t="n">
-        <v>32</v>
+        <v>15.5</v>
       </c>
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr"/>
@@ -7792,26 +7788,26 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Lay 0x3</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>PARAGUAY CUP</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Sol de America</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Sportivo Trinidense</t>
+          <t>Coventry</t>
         </is>
       </c>
       <c r="F208" t="n">
-        <v>32</v>
+        <v>11.5</v>
       </c>
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr"/>
@@ -7824,26 +7820,26 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>ROMANIA 2</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Unirea Slobozia</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>FC Metaloglobus Bucuresti</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="F209" t="n">
-        <v>18.5</v>
+        <v>15</v>
       </c>
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr"/>
@@ -7856,26 +7852,26 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Al-Taawoun Buraidah</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Al-Feiha</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F210" t="n">
-        <v>18.5</v>
+        <v>29</v>
       </c>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr"/>
@@ -7888,7 +7884,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -7898,16 +7894,16 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Cambridge Utd</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Leyton Orient</t>
         </is>
       </c>
       <c r="F211" t="n">
-        <v>17.5</v>
+        <v>32</v>
       </c>
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr"/>
@@ -7920,26 +7916,26 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Lay 2x2</t>
+          <t>Lay 0x3</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>PARAGUAY CUP</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Fleetwood Town</t>
+          <t>Sol de America</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Shrewsbury</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F212" t="n">
-        <v>19.5</v>
+        <v>32</v>
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr"/>
@@ -7957,21 +7953,21 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>ROMANIA 2</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Unirea Slobozia</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>FC Metaloglobus Bucuresti</t>
         </is>
       </c>
       <c r="F213" t="n">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr"/>
@@ -7989,17 +7985,17 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>ENGLAND CUP</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Stoke</t>
+          <t>Al-Taawoun Buraidah</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Hull</t>
+          <t>Al-Feiha</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -8026,12 +8022,12 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Cambridge Utd</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Leyton Orient</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="F215" t="n">
@@ -8058,16 +8054,16 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Nottm Forest</t>
+          <t>Fleetwood Town</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Shrewsbury</t>
         </is>
       </c>
       <c r="F216" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr"/>
@@ -8085,21 +8081,21 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>PARAGUAY CUP</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>General Caballero</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Rubio Nu</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="F217" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr"/>
@@ -8117,24 +8113,152 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>SPAIN 1</t>
+          <t>ENGLAND CUP</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Stoke</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Hull</t>
         </is>
       </c>
       <c r="F218" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>ENGLAND CUP</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Walsall</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Leyton Orient</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>ENGLAND CUP</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Nottm Forest</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>18</v>
+      </c>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>PARAGUAY CUP</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>General Caballero</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Rubio Nu</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>18</v>
+      </c>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Lay 2x2</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>SPAIN 1</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Valencia</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Betis</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>18</v>
+      </c>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: sincronizar repositorio completo, forward oculto, planilhas corrigidas com odds reais da Betfair e paineis Streamlit
</commit_message>
<xml_diff>
--- a/placares_manuais.xlsx
+++ b/placares_manuais.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M487"/>
+  <dimension ref="A1:M482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19876,7 +19876,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
@@ -19886,21 +19886,21 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ARGENTINA CUP</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Velez Sarsfield</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="F460" t="n">
-        <v>11.5</v>
+        <v>10</v>
       </c>
       <c r="G460" t="inlineStr"/>
       <c r="H460" t="inlineStr"/>
@@ -19913,7 +19913,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -19923,21 +19923,21 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>ENGLAND 2</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Bandirmaspor</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>Antalyaspor</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="F461" t="n">
-        <v>11</v>
+        <v>13.5</v>
       </c>
       <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr"/>
@@ -19950,7 +19950,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -19960,21 +19960,21 @@
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>ARGENTINA CUP</t>
         </is>
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Umraniyespor</t>
+          <t>Velez Sarsfield</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>Muglaspor</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="F462" t="n">
-        <v>9.4</v>
+        <v>8</v>
       </c>
       <c r="G462" t="inlineStr"/>
       <c r="H462" t="inlineStr"/>
@@ -19987,7 +19987,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -19997,21 +19997,21 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="F463" t="n">
-        <v>11</v>
+        <v>9.4</v>
       </c>
       <c r="G463" t="inlineStr"/>
       <c r="H463" t="inlineStr"/>
@@ -20024,31 +20024,31 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>ENGLAND 4</t>
+          <t>BOSNIA 1</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>Cheltenham</t>
+          <t>Borac Banja Luka</t>
         </is>
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Zeljeznicar</t>
         </is>
       </c>
       <c r="F464" t="n">
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="G464" t="inlineStr"/>
       <c r="H464" t="inlineStr"/>
@@ -20061,31 +20061,31 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>ENGLAND 4</t>
+          <t>ENGLAND 2</t>
         </is>
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Swindon</t>
+          <t>West Brom</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Port Vale</t>
+          <t>Charlton</t>
         </is>
       </c>
       <c r="F465" t="n">
-        <v>10.5</v>
+        <v>8.4</v>
       </c>
       <c r="G465" t="inlineStr"/>
       <c r="H465" t="inlineStr"/>
@@ -20098,31 +20098,31 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>Lay 0x1</t>
+          <t>Lay 1x0</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>ENGLAND 3</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Barnsley</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Blackpool</t>
         </is>
       </c>
       <c r="F466" t="n">
-        <v>8.800000000000001</v>
+        <v>12.5</v>
       </c>
       <c r="G466" t="inlineStr"/>
       <c r="H466" t="inlineStr"/>
@@ -20135,31 +20135,31 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>SCOTLAND 1</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>Umraniyespor</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Muglaspor</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="F467" t="n">
-        <v>9.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="G467" t="inlineStr"/>
       <c r="H467" t="inlineStr"/>
@@ -20172,31 +20172,31 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>SCOTLAND 1</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>Dundee Utd</t>
         </is>
       </c>
       <c r="F468" t="n">
-        <v>8.800000000000001</v>
+        <v>14.5</v>
       </c>
       <c r="G468" t="inlineStr"/>
       <c r="H468" t="inlineStr"/>
@@ -20209,31 +20209,31 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 2x0</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>ENGLAND 4</t>
+          <t>ENGLAND 3</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Chesterfield</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Gillingham</t>
+          <t>Mansfield</t>
         </is>
       </c>
       <c r="F469" t="n">
-        <v>8.199999999999999</v>
+        <v>14.5</v>
       </c>
       <c r="G469" t="inlineStr"/>
       <c r="H469" t="inlineStr"/>
@@ -20246,31 +20246,31 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Lay 1x0</t>
+          <t>Lay 0x2</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>BRAZIL 2</t>
+          <t>SCOTLAND 1</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Falkirk</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Rangers</t>
         </is>
       </c>
       <c r="F470" t="n">
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="G470" t="inlineStr"/>
       <c r="H470" t="inlineStr"/>
@@ -20283,7 +20283,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
@@ -20293,21 +20293,21 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>Boluspor</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>Keciorengucu</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="F471" t="n">
-        <v>11.5</v>
+        <v>16</v>
       </c>
       <c r="G471" t="inlineStr"/>
       <c r="H471" t="inlineStr"/>
@@ -20320,7 +20320,7 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
@@ -20330,17 +20330,17 @@
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>ENGLAND 4</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>Accrington</t>
+          <t>Van Buyuksehir Belediyespor</t>
         </is>
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>Grimsby</t>
+          <t>Batman Petrolspor</t>
         </is>
       </c>
       <c r="F472" t="n">
@@ -20357,7 +20357,7 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
@@ -20367,21 +20367,21 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>ENGLAND 4</t>
+          <t>ARGENTINA CUP</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>Cheltenham</t>
+          <t>Velez Sarsfield</t>
         </is>
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="F473" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G473" t="inlineStr"/>
       <c r="H473" t="inlineStr"/>
@@ -20394,7 +20394,7 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
@@ -20404,17 +20404,17 @@
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>TURKEY 2</t>
+          <t>SAUDI ARABIA 1</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>Bandirmaspor</t>
+          <t>Hajer Club</t>
         </is>
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>Antalyaspor</t>
+          <t>Al-Anwar Club</t>
         </is>
       </c>
       <c r="F474" t="n">
@@ -20431,7 +20431,7 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
@@ -20441,21 +20441,21 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>CZECH 1</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Al Jeel</t>
+          <t>FC Zbrojovka Brno</t>
         </is>
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>Jeddah Club</t>
+          <t>Hradec Kralove</t>
         </is>
       </c>
       <c r="F475" t="n">
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="G475" t="inlineStr"/>
       <c r="H475" t="inlineStr"/>
@@ -20468,7 +20468,7 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
@@ -20478,21 +20478,21 @@
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>TURKEY 2</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>Al Orubah</t>
+          <t>Fatih Karagumruk Istanbul</t>
         </is>
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Al-Zulfi SC</t>
+          <t>Kayserispor</t>
         </is>
       </c>
       <c r="F476" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G476" t="inlineStr"/>
       <c r="H476" t="inlineStr"/>
@@ -20505,7 +20505,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -20520,16 +20520,16 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Sariyer G.K.</t>
+          <t>Sivasspor</t>
         </is>
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Pendikspor</t>
+          <t>Mardin Buyuksehir Belediyespor</t>
         </is>
       </c>
       <c r="F477" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G477" t="inlineStr"/>
       <c r="H477" t="inlineStr"/>
@@ -20542,7 +20542,7 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -20552,21 +20552,21 @@
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA 1</t>
+          <t>CZECH 1</t>
         </is>
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>Al Najma Club</t>
+          <t>Bohemians 1905</t>
         </is>
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>Al Jabalain</t>
+          <t>FK Jablonec</t>
         </is>
       </c>
       <c r="F478" t="n">
-        <v>19.5</v>
+        <v>18</v>
       </c>
       <c r="G478" t="inlineStr"/>
       <c r="H478" t="inlineStr"/>
@@ -20579,7 +20579,7 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -20594,16 +20594,16 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Lincoln</t>
+          <t>Millwall</t>
         </is>
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Blackburn</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="F479" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
       <c r="G479" t="inlineStr"/>
       <c r="H479" t="inlineStr"/>
@@ -20616,7 +20616,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -20626,21 +20626,21 @@
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>ENGLAND 3</t>
         </is>
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Burton Albion</t>
         </is>
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>Derby</t>
+          <t>AFC Wimbledon</t>
         </is>
       </c>
       <c r="F480" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G480" t="inlineStr"/>
       <c r="H480" t="inlineStr"/>
@@ -20653,7 +20653,7 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -20663,21 +20663,21 @@
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>PARAGUAY 1</t>
         </is>
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Preston</t>
+          <t>Club Sportivo Ameliano</t>
         </is>
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Sportivo Trinidense</t>
         </is>
       </c>
       <c r="F481" t="n">
-        <v>16.5</v>
+        <v>18</v>
       </c>
       <c r="G481" t="inlineStr"/>
       <c r="H481" t="inlineStr"/>
@@ -20690,7 +20690,7 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
@@ -20700,21 +20700,21 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>ENGLAND 2</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Watford</t>
+          <t>Millonarios</t>
         </is>
       </c>
       <c r="F482" t="n">
-        <v>18.5</v>
+        <v>20</v>
       </c>
       <c r="G482" t="inlineStr"/>
       <c r="H482" t="inlineStr"/>
@@ -20724,191 +20724,6 @@
       <c r="L482" t="inlineStr"/>
       <c r="M482" t="inlineStr"/>
     </row>
-    <row r="483">
-      <c r="A483" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B483" t="inlineStr">
-        <is>
-          <t>Lay 2x2</t>
-        </is>
-      </c>
-      <c r="C483" t="inlineStr">
-        <is>
-          <t>ENGLAND 3</t>
-        </is>
-      </c>
-      <c r="D483" t="inlineStr">
-        <is>
-          <t>Bromley</t>
-        </is>
-      </c>
-      <c r="E483" t="inlineStr">
-        <is>
-          <t>Leyton Orient</t>
-        </is>
-      </c>
-      <c r="F483" t="n">
-        <v>18</v>
-      </c>
-      <c r="G483" t="inlineStr"/>
-      <c r="H483" t="inlineStr"/>
-      <c r="I483" t="inlineStr"/>
-      <c r="J483" t="inlineStr"/>
-      <c r="K483" t="inlineStr"/>
-      <c r="L483" t="inlineStr"/>
-      <c r="M483" t="inlineStr"/>
-    </row>
-    <row r="484">
-      <c r="A484" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B484" t="inlineStr">
-        <is>
-          <t>Lay 2x2</t>
-        </is>
-      </c>
-      <c r="C484" t="inlineStr">
-        <is>
-          <t>ENGLAND 3</t>
-        </is>
-      </c>
-      <c r="D484" t="inlineStr">
-        <is>
-          <t>Peterborough</t>
-        </is>
-      </c>
-      <c r="E484" t="inlineStr">
-        <is>
-          <t>Stevenage</t>
-        </is>
-      </c>
-      <c r="F484" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="G484" t="inlineStr"/>
-      <c r="H484" t="inlineStr"/>
-      <c r="I484" t="inlineStr"/>
-      <c r="J484" t="inlineStr"/>
-      <c r="K484" t="inlineStr"/>
-      <c r="L484" t="inlineStr"/>
-      <c r="M484" t="inlineStr"/>
-    </row>
-    <row r="485">
-      <c r="A485" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B485" t="inlineStr">
-        <is>
-          <t>Lay 2x2</t>
-        </is>
-      </c>
-      <c r="C485" t="inlineStr">
-        <is>
-          <t>ENGLAND 4</t>
-        </is>
-      </c>
-      <c r="D485" t="inlineStr">
-        <is>
-          <t>Rochdale</t>
-        </is>
-      </c>
-      <c r="E485" t="inlineStr">
-        <is>
-          <t>Shrewsbury</t>
-        </is>
-      </c>
-      <c r="F485" t="n">
-        <v>18</v>
-      </c>
-      <c r="G485" t="inlineStr"/>
-      <c r="H485" t="inlineStr"/>
-      <c r="I485" t="inlineStr"/>
-      <c r="J485" t="inlineStr"/>
-      <c r="K485" t="inlineStr"/>
-      <c r="L485" t="inlineStr"/>
-      <c r="M485" t="inlineStr"/>
-    </row>
-    <row r="486">
-      <c r="A486" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B486" t="inlineStr">
-        <is>
-          <t>Lay 2x2</t>
-        </is>
-      </c>
-      <c r="C486" t="inlineStr">
-        <is>
-          <t>ENGLAND 4</t>
-        </is>
-      </c>
-      <c r="D486" t="inlineStr">
-        <is>
-          <t>Tranmere</t>
-        </is>
-      </c>
-      <c r="E486" t="inlineStr">
-        <is>
-          <t>Rotherham</t>
-        </is>
-      </c>
-      <c r="F486" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="G486" t="inlineStr"/>
-      <c r="H486" t="inlineStr"/>
-      <c r="I486" t="inlineStr"/>
-      <c r="J486" t="inlineStr"/>
-      <c r="K486" t="inlineStr"/>
-      <c r="L486" t="inlineStr"/>
-      <c r="M486" t="inlineStr"/>
-    </row>
-    <row r="487">
-      <c r="A487" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B487" t="inlineStr">
-        <is>
-          <t>Lay 2x2</t>
-        </is>
-      </c>
-      <c r="C487" t="inlineStr">
-        <is>
-          <t>PERU 1</t>
-        </is>
-      </c>
-      <c r="D487" t="inlineStr">
-        <is>
-          <t>Atletico Grau</t>
-        </is>
-      </c>
-      <c r="E487" t="inlineStr">
-        <is>
-          <t>Melgar</t>
-        </is>
-      </c>
-      <c r="F487" t="n">
-        <v>19</v>
-      </c>
-      <c r="G487" t="inlineStr"/>
-      <c r="H487" t="inlineStr"/>
-      <c r="I487" t="inlineStr"/>
-      <c r="J487" t="inlineStr"/>
-      <c r="K487" t="inlineStr"/>
-      <c r="L487" t="inlineStr"/>
-      <c r="M487" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>